<commit_message>
Condense ALM checklist to 6 acceptance criteria
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149r7b5293oK3v6EmbinnuA
</commit_message>
<xml_diff>
--- a/TTZV-6011_ALM_Check_list.xlsx
+++ b/TTZV-6011_ALM_Check_list.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="92.85546875" customWidth="1" style="2" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="3" ht="66" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Պարտատոմսի հաշիվը ներառված է PLUS CLUB, PLUS DIGITAL, STATUS փաթեթների միջին մնացորդի հաշվարկում՝ ցպահանջ և ժամկետային ավանդային հաշիվների հետ միասին (միջին մնացորդ = ցպահանջ + ժամկետային + պարտատոմսի հաշիվների եռամսյակային միջին մնացորդների գումար):</t>
+          <t>PLUS CLUB, PLUS DIGITAL, STATUS փաթեթների միջին մնացորդի հաշվարկում ներառված է հաճախորդի պարտատոմսի հաշիվը՝ ցպահանջ և ժամկետային ավանդային հաշիվների հետ միասին: Պարտատոմսը հաշվառվում է անվանական արժեքով, իսկ Քայլ 1-ի և Քայլ 2-ի ստուգումները կատարվում են եռամսյակային միջին մնացորդով:</t>
         </is>
       </c>
       <c r="B3" s="8" t="n"/>
@@ -528,33 +528,37 @@
     <row r="4" ht="66" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Պարտատոմսի հաշվի մնացորդը հաշվառվում է անվանական արժեքով: Ձեռքբերման / շուկայական արժեքը և կուտակված արժեկտրոնը չեն դիտարկվում:
-Օրինակ՝ ավանդներ 1,000,000 + պարտատոմս (անվանական 1,000,000, ձեռքբերման արժեք 980,000) → միջին մնացորդ 2,000,000:</t>
+          <t>PLUS CLUB.
+- ավանդներ 1,500,000 + պարտատոմս 1,000,000 → սպասարկման վճար 5,000 ՀՀԴ (առանց պարտատոմսի՝ 10,000 ՀՀԴ)
+- ավանդներ 3,000,000 + պարտատոմս 2,500,000 → սպասարկման վճար 0 ՀՀԴ</t>
         </is>
       </c>
       <c r="B4" s="8" t="n"/>
     </row>
-    <row r="5" ht="33" customHeight="1">
+    <row r="5" ht="66" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Փաթեթի որակավորման (Քայլ 1) և սպասարկման վճարի որոշման (Քայլ 2) ստուգումները կատարվում են եռամսյակային միջին մնացորդով, որում ներառված է պարտատոմսի հաշիվը:</t>
+          <t>PLUS DIGITAL.
+- ավանդներ 1,500,000 + պարտատոմս 1,000,000 → սպասարկման վճար 2,000 ՀՀԴ (առանց պարտատոմսի՝ 7,000 ՀՀԴ)
+- ավանդներ 3,000,000 + պարտատոմս 2,500,000 → սպասարկման վճար 0 ՀՀԴ</t>
         </is>
       </c>
       <c r="B5" s="8" t="n"/>
     </row>
-    <row r="6" ht="49.5" customHeight="1">
+    <row r="6" ht="66" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Եթե հաճախորդն ունի միայն պարտատոմսի հաշիվ (ավանդային հաշիվներ չկան), միջին մնացորդը հաշվարկվում է պարտատոմսի հաշվի մնացորդով:
-Օրինակ՝ PLUS CLUB, պարտատոմս 2,500,000 → Քայլ 2 → 5,000 ՀՀԴ:</t>
+          <t>STATUS.
+- ավանդներ 15,000,000 + պարտատոմս 6,000,000 → սպասարկման վճար 10,000 ՀՀԴ, հաճախորդը չի ներառվում անհամապատասխան հաճախորդների ցուցակում
+- ավանդներ 25,000,000 + պարտատոմս 20,000,000 → սպասարկման վճար 0 ՀՀԴ</t>
         </is>
       </c>
       <c r="B6" s="8" t="n"/>
     </row>
-    <row r="7" ht="16.5" customHeight="1">
+    <row r="7" ht="49.5" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Հաճախորդի բոլոր պարտատոմսի հաշիվների մնացորդները գումարվում են:</t>
+          <t>LSoft-ում սպասարկման վճարը գանձվում է ճիշտ գումարով՝ ամսվա 1-ին աշխատանքային օրը: Պարտատոմսի շնորհիվ որակավորված հաճախորդները չեն ներառվում ՍԾՎ/ՍԾԶՎ-ին տրամադրվող անհամապատասխան հաճախորդների ցուցակում և ծանուցում չեն ստանում:</t>
         </is>
       </c>
       <c r="B7" s="8" t="n"/>
@@ -562,171 +566,18 @@
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Զրոյական մնացորդով կամ փակված պարտատոմսի հաշիվը չի ազդում հաշվարկի արդյունքի վրա և սխալ չի առաջացնում:</t>
+          <t>Առանց պարտատոմսի հաշվի հաճախորդների, ինչպես նաև այլ փաթեթների հաշվարկի արդյունքները չեն փոխվել:</t>
         </is>
       </c>
       <c r="B8" s="8" t="n"/>
     </row>
-    <row r="9" ht="33" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Միջին մնացորդի հաշվարկում ներառվում են միայն տվյալ հաճախորդի սեփական պարտատոմսի հաշիվները. այլ հաճախորդի պարտատոմսի հաշիվը չի ներառվում:</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="49.5" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>PLUS CLUB. ավանդներ 1,500,000 + պարտատոմս 1,000,000 (միջին մնացորդ 2,500,000, աշխատավարձ չկա) → Քայլ 1-ը բավարարված է, Քայլ 2 → սպասարկման վճար 5,000 ՀՀԴ (առանց պարտատոմսի կլիներ Քայլ 3 → 10,000 ՀՀԴ):</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>PLUS CLUB. ավանդներ 3,000,000 + պարտատոմս 2,500,000 (միջին մնացորդ 5,500,000) → սպասարկման վճար 0 ՀՀԴ:</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="49.5" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>PLUS DIGITAL. ավանդներ 1,500,000 + պարտատոմս 1,000,000 (միջին մնացորդ 2,500,000, աշխատավարձ չկա) → Քայլ 2 → սպասարկման վճար 2,000 ՀՀԴ (առանց պարտատոմսի կլիներ Քայլ 3 → 7,000 ՀՀԴ):</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="33" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>PLUS DIGITAL. ավանդներ 3,000,000 + պարտատոմս 2,500,000 (միջին մնացորդ 5,500,000) → սպասարկման վճար 0 ՀՀԴ:</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n"/>
-    </row>
-    <row r="14" ht="49.5" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>STATUS. ավանդներ 15,000,000 + պարտատոմս 6,000,000 (միջին մնացորդ 21,000,000) → Քայլ 2 → սպասարկման վճար 10,000 ՀՀԴ, հաճախորդը չի ներառվում ՍԾՎ/ՍԾԶՎ-ին տրամադրվող անհամապատասխան հաճախորդների ցուցակում:</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="33" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>STATUS. ավանդներ 25,000,000 + պարտատոմս 20,000,000 (միջին մնացորդ 45,000,000) → սպասարկման վճար 0 ՀՀԴ:</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="49.5" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>PLUS CLUB / PLUS DIGITAL. աշխատավարձով որակավորված հաճախորդի (աշխատավարձ ≥ 400,000) Քայլ 2-ի ստուգման մեջ ևս ներառվում է պարտատոմսը. ավանդներ 2,000,000 + պարտատոմս 3,500,000 → 0 ՀՀԴ:</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="49.5" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>PLUS CLUB / PLUS DIGITAL. եթե պարտատոմսով հանդերձ միջին մնացորդը &lt; 2,000,000 է (օր.՝ ավանդներ 500,000 + պարտատոմս 1,000,000), հաճախորդն անցնում է Քայլ 3՝ գործող տրամաբանությամբ (5,000 / 2,000 ՀՀԴ կամ 10,000 / 7,000 ՀՀԴ):</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n"/>
-    </row>
-    <row r="18" ht="49.5" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Շեմային արժեքներ (պայմանը՝ ≥). PLUS CLUB / PLUS DIGITAL՝ 2,000,000 (որակավորվում է) / 1,999,999 (չի որակավորվում), 5,000,000 (0 ՀՀԴ) / 4,999,999 (5,000 / 2,000 ՀՀԴ):</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n"/>
-    </row>
-    <row r="19" ht="49.5" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Շեմային արժեքներ (պայմանը՝ ≥). STATUS՝ 20,000,000 (10,000 ՀՀԴ, ցուցակում չէ) / 19,999,999 (10,000 ՀՀԴ, ներառվում է ցուցակում), 40,000,000 (0 ՀՀԴ) / 39,999,999 (10,000 ՀՀԴ):</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n"/>
-    </row>
-    <row r="20" ht="33" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>LSoft-ում սպասարկման վճարը գանձվում է ճիշտ գումարով, ճիշտ հաշվից, ամսվա 1-ին աշխատանքային օրը, առանց կրկնակի գանձման:</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="49.5" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>STATUS. ՍԾՎ/ՍԾԶՎ-ին տրամադրվող անհամապատասխան հաճախորդների ցուցակում ներառված են միայն այն հաճախորդները, որոնք պարտատոմսը հաշվի առնելով էլ չեն համապատասխանում չափանիշներին:</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="33" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>PLUS CLUB / PLUS DIGITAL. պարտատոմսի շնորհիվ որակավորված հաճախորդները անհամապատասխանության ծանուցում չեն ստանում և չեն ներառվում ՍԾԶՎ-ին տրամադրվող ցուցակում:</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="n"/>
-    </row>
-    <row r="23" ht="33" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Առանց պարտատոմսի հաշվի հաճախորդների համար հաշվարկի արդյունքները (վճար, ցուցակ, ծանուցում) չեն փոխվել TTZV-4447 / LSBANK-994 լուծման համեմատ:</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="n"/>
-    </row>
-    <row r="24" ht="33" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Աշխատավարձի և դրան հավասարեցված եկամտի չափանիշի ստուգումը չի փոխվել. պարտատոմսի մարումը / արժեկտրոնը աշխատավարձ չի համարվում:</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n"/>
-    </row>
-    <row r="25" ht="33" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Optimal, Advanced և այլ փաթեթների, ինչպես նաև առանց փաթեթի հաճախորդների հաշվարկը չի փոխվել:</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-    </row>
-    <row r="26" ht="33" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Մեկ փաթեթի սակագնի փոփոխությունը կիրառվում է միայն տվյալ փաթեթի վրա, պարտատոմսի ներառումը շարունակում է աշխատել:</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-    </row>
-    <row r="27" ht="33" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Ամսական հաշվարկը բոլոր փաթեթային հաճախորդների համար գործարկվում է ամսվա 1-ին աշխատանքային օրը և ավարտվում է առանց սխալների:</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="n"/>
-    </row>
-    <row r="28" ht="33" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Պարտատոմս ունեցող հաճախորդների նմուշի (յուրաքանչյուր փաթեթից) համար ձեռքով հաշվարկված միջին մնացորդը և սպասարկման վճարը համընկնում են համակարգի արդյունքի հետ:</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="n"/>
-    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>